<commit_message>
Update to use new job adverts data instead of snapshots due to ONS pausing publication of the snapshot data. Also includes an update to the latest (November 2025) online job adverts data.
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jevans8\Repos\lsip_dashboard\Data\3-1_DataTable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmehta4\Repos\lsip_dashboard\Data\3-1_DataTable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91CA5E8E-A54C-4860-B017-C7DC9575D383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21EFB29-6388-4B1D-AFC4-15AAA8E0DF71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -119,9 +119,6 @@
     <t>Jul 2024 - Jun 2025 (14/10/25)</t>
   </si>
   <si>
-    <t>Jul 2025 (29/08/25)</t>
-  </si>
-  <si>
     <t>Mar 2025 (14/10/24)</t>
   </si>
   <si>
@@ -143,9 +140,6 @@
     <t>Oct 2024 - Sep 2025 (20/01/26)</t>
   </si>
   <si>
-    <t>TBC*</t>
-  </si>
-  <si>
     <t>Dec 2023 - Dec 2024 (20/11/25)</t>
   </si>
   <si>
@@ -162,6 +156,12 @@
   </si>
   <si>
     <t>Aug 2025 – Jul 2026 (Nov 26)</t>
+  </si>
+  <si>
+    <t>Nov 2025 (23/12/25)</t>
+  </si>
+  <si>
+    <t>Dec 2025 (Jan 26)</t>
   </si>
 </sst>
 </file>
@@ -571,7 +571,7 @@
         <v>26</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="125" customHeight="1" x14ac:dyDescent="0.35">
@@ -585,7 +585,7 @@
         <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -599,7 +599,7 @@
         <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.35">
@@ -607,13 +607,13 @@
         <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" t="s">
         <v>38</v>
       </c>
-      <c r="C5" t="s">
-        <v>40</v>
-      </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -621,13 +621,13 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" t="s">
         <v>39</v>
-      </c>
-      <c r="C6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -652,10 +652,10 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" t="s">
         <v>28</v>
-      </c>
-      <c r="D8" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -666,10 +666,10 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
         <v>28</v>
-      </c>
-      <c r="D9" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -680,10 +680,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -691,13 +691,13 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -705,13 +705,13 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -722,10 +722,10 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="D13" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Rerun code to update to latest APS employment data. Update data table and data text to reflect new data. Run shiny tests
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmehta4\Repos\lsip_dashboard\Data\3-1_DataTable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjames2\OneDrive - Department for Education\Documents\RProjects\lsip_dashboard\Data\3-1_DataTable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21EFB29-6388-4B1D-AFC4-15AAA8E0DF71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D75A151-E2FF-4B82-93EE-270BCC805CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
+    <workbookView xWindow="1900" yWindow="740" windowWidth="20660" windowHeight="14300" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t>Data​</t>
   </si>
@@ -114,9 +114,6 @@
   </si>
   <si>
     <t>Jan 2025 - Dec 2025 (Apr 26)</t>
-  </si>
-  <si>
-    <t>Jul 2024 - Jun 2025 (14/10/25)</t>
   </si>
   <si>
     <t>Mar 2025 (14/10/24)</t>
@@ -568,10 +565,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="125" customHeight="1" x14ac:dyDescent="0.35">
@@ -582,10 +579,10 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -596,10 +593,10 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.35">
@@ -607,13 +604,13 @@
         <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s">
         <v>38</v>
-      </c>
-      <c r="D5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -621,13 +618,13 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
         <v>37</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>38</v>
-      </c>
-      <c r="D6" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -652,10 +649,10 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
         <v>27</v>
-      </c>
-      <c r="D8" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -666,10 +663,10 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
         <v>27</v>
-      </c>
-      <c r="D9" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -680,10 +677,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" t="s">
         <v>34</v>
-      </c>
-      <c r="D10" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -691,13 +688,13 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -705,13 +702,13 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -722,10 +719,10 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" t="s">
         <v>40</v>
-      </c>
-      <c r="D13" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Correct the link for KS4 and KS5. Update the date for FE data on the data sources.
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjames2\OneDrive - Department for Education\Documents\RProjects\lsip_dashboard\Data\3-1_DataTable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D75A151-E2FF-4B82-93EE-270BCC805CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{1D75A151-E2FF-4B82-93EE-270BCC805CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87491967-A868-4943-8D07-3B402C63C8CD}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="740" windowWidth="20660" windowHeight="14300" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -131,9 +131,6 @@
     <t>Aug 2023 -  Jul 2024 (22/23 learners) (16/10/25)</t>
   </si>
   <si>
-    <t>Aug 2023 -  Jul 2024 (22/23 learners) (Feb 26)</t>
-  </si>
-  <si>
     <t>Oct 2024 - Sep 2025 (20/01/26)</t>
   </si>
   <si>
@@ -158,7 +155,10 @@
     <t>Nov 2025 (23/12/25)</t>
   </si>
   <si>
-    <t>Dec 2025 (Jan 26)</t>
+    <t>Aug 2023 -  Jul 2024 (22/23 learners) (Mar 26)</t>
+  </si>
+  <si>
+    <t>Jan 2025 (Feb 26)</t>
   </si>
 </sst>
 </file>
@@ -565,7 +565,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
         <v>25</v>
@@ -579,7 +579,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
         <v>25</v>
@@ -593,7 +593,7 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D4" t="s">
         <v>25</v>
@@ -604,13 +604,13 @@
         <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" t="s">
         <v>37</v>
-      </c>
-      <c r="D5" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -618,13 +618,13 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
         <v>36</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>37</v>
-      </c>
-      <c r="D6" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -677,10 +677,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" t="s">
         <v>33</v>
-      </c>
-      <c r="D10" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -694,7 +694,7 @@
         <v>30</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -708,7 +708,7 @@
         <v>30</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -719,7 +719,7 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D13" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
Update to latest online job ad data
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjames2\OneDrive - Department for Education\Documents\RProjects\lsip_dashboard\Data\3-1_DataTable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{1D75A151-E2FF-4B82-93EE-270BCC805CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87491967-A868-4943-8D07-3B402C63C8CD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3EE8CEB-6D67-456F-ADBE-A57DA970F725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
@@ -152,13 +152,13 @@
     <t>Aug 2025 – Jul 2026 (Nov 26)</t>
   </si>
   <si>
-    <t>Nov 2025 (23/12/25)</t>
-  </si>
-  <si>
     <t>Aug 2023 -  Jul 2024 (22/23 learners) (Mar 26)</t>
   </si>
   <si>
-    <t>Jan 2025 (Feb 26)</t>
+    <t>Jan 2026 (27/02/26)</t>
+  </si>
+  <si>
+    <t>Feb 2026 (Mar 26)</t>
   </si>
 </sst>
 </file>
@@ -694,7 +694,7 @@
         <v>30</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -708,7 +708,7 @@
         <v>30</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -719,7 +719,7 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D13" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
Updated ONS job adverts data and KS4 and KS5 destinations data.
Also minor updates to account for the job adverts page.
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pjames2\OneDrive - Department for Education\Documents\RProjects\lsip_dashboard\Data\3-1_DataTable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmehta4\Repos\lsip_dashboard\Data\3-1_DataTable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3EE8CEB-6D67-456F-ADBE-A57DA970F725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{397B93E5-4144-499E-918B-2CB87CFF9ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -128,9 +128,6 @@
     <t>&lt;a href = 'https://explore-education-statistics.service.gov.uk/find-statistics/key-stage-4-destination-measures/'&gt;Key stage 4 destination measures&lt;/a&gt;</t>
   </si>
   <si>
-    <t>Aug 2023 -  Jul 2024 (22/23 learners) (16/10/25)</t>
-  </si>
-  <si>
     <t>Oct 2024 - Sep 2025 (20/01/26)</t>
   </si>
   <si>
@@ -155,10 +152,13 @@
     <t>Aug 2023 -  Jul 2024 (22/23 learners) (Mar 26)</t>
   </si>
   <si>
-    <t>Jan 2026 (27/02/26)</t>
-  </si>
-  <si>
-    <t>Feb 2026 (Mar 26)</t>
+    <t>Feb 2026 (30/03/26)</t>
+  </si>
+  <si>
+    <t>Mar 2026 (24/04/26)</t>
+  </si>
+  <si>
+    <t>Aug 2023 -  Jul 2024 (22/23 learners) (26/03/26)</t>
   </si>
 </sst>
 </file>
@@ -565,7 +565,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
         <v>25</v>
@@ -579,7 +579,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
         <v>25</v>
@@ -593,7 +593,7 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
         <v>25</v>
@@ -604,13 +604,13 @@
         <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" t="s">
         <v>36</v>
-      </c>
-      <c r="D5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -618,13 +618,13 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
         <v>35</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>36</v>
-      </c>
-      <c r="D6" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -677,10 +677,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" t="s">
         <v>32</v>
-      </c>
-      <c r="D10" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -691,10 +691,10 @@
         <v>29</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -705,10 +705,10 @@
         <v>28</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -719,10 +719,10 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" t="s">
         <v>39</v>
-      </c>
-      <c r="D13" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Updated importDestinations.R script to fix issue caused by updated LADs to regions mapping in destinations data.
Also corrected typos in various scripts.
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmehta4\Repos\lsip_dashboard\Data\3-1_DataTable\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{397B93E5-4144-499E-918B-2CB87CFF9ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
@@ -149,9 +149,6 @@
     <t>Aug 2025 – Jul 2026 (Nov 26)</t>
   </si>
   <si>
-    <t>Aug 2023 -  Jul 2024 (22/23 learners) (Mar 26)</t>
-  </si>
-  <si>
     <t>Feb 2026 (30/03/26)</t>
   </si>
   <si>
@@ -159,6 +156,9 @@
   </si>
   <si>
     <t>Aug 2023 -  Jul 2024 (22/23 learners) (26/03/26)</t>
+  </si>
+  <si>
+    <t>Aug 2023 -  Jul 2024 (22/23 learners) (tbc)</t>
   </si>
 </sst>
 </file>
@@ -691,10 +691,10 @@
         <v>29</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -705,10 +705,10 @@
         <v>28</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -719,10 +719,10 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" t="s">
         <v>38</v>
-      </c>
-      <c r="D13" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -743,5 +743,15 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;11&amp;K000000 OFFICIAL - FOR PUBLIC RELEASE&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;11&amp;K000000 OFFICIAL - FOR PUBLIC RELEASE</oddFooter>
+  </headerFooter>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{dbf2ff9d-e249-40e2-b463-0b922d4f2f25}" enabled="1" method="Privileged" siteId="{fad277c9-c60a-4da1-b5f3-b3b8b34a82f9}" contentBits="3" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Clean renv Update version control and data tables Update APS data (including qualifications)
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmehta4\Repos\lsip_dashboard\Data\3-1_DataTable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC9CCE9B-45FD-4B0A-AACC-A7C0A0466434}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
   <si>
     <t>Data​</t>
   </si>
@@ -110,9 +110,6 @@
     <t>2035 (05/08/24)</t>
   </si>
   <si>
-    <t>Jan 2024 - Dec 2024 (15/04/25)</t>
-  </si>
-  <si>
     <t>Jan 2025 - Dec 2025 (Apr 26)</t>
   </si>
   <si>
@@ -128,9 +125,6 @@
     <t>&lt;a href = 'https://explore-education-statistics.service.gov.uk/find-statistics/key-stage-4-destination-measures/'&gt;Key stage 4 destination measures&lt;/a&gt;</t>
   </si>
   <si>
-    <t>Oct 2024 - Sep 2025 (20/01/26)</t>
-  </si>
-  <si>
     <t>Dec 2023 - Dec 2024 (20/11/25)</t>
   </si>
   <si>
@@ -159,6 +153,9 @@
   </si>
   <si>
     <t>Aug 2023 -  Jul 2024 (22/23 learners) (tbc)</t>
+  </si>
+  <si>
+    <t>April 2025 - Mar 2026 (TBC)</t>
   </si>
 </sst>
 </file>
@@ -565,10 +562,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="125" customHeight="1" x14ac:dyDescent="0.35">
@@ -579,10 +576,10 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -593,10 +590,10 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.35">
@@ -604,13 +601,13 @@
         <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
         <v>33</v>
       </c>
-      <c r="C5" t="s">
-        <v>35</v>
-      </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -618,13 +615,13 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
         <v>34</v>
-      </c>
-      <c r="C6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -638,7 +635,7 @@
         <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -649,10 +646,10 @@
         <v>10</v>
       </c>
       <c r="C8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" t="s">
         <v>26</v>
-      </c>
-      <c r="D8" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -663,10 +660,10 @@
         <v>10</v>
       </c>
       <c r="C9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" t="s">
         <v>26</v>
-      </c>
-      <c r="D9" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -677,10 +674,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -688,13 +685,13 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -702,13 +699,13 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -719,10 +716,10 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Update job ad data to April 2026
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC9CCE9B-45FD-4B0A-AACC-A7C0A0466434}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7D70FA9-1DA0-472D-9218-E1429AD6A4EA}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
@@ -143,12 +143,6 @@
     <t>Aug 2025 – Jul 2026 (Nov 26)</t>
   </si>
   <si>
-    <t>Feb 2026 (30/03/26)</t>
-  </si>
-  <si>
-    <t>Mar 2026 (24/04/26)</t>
-  </si>
-  <si>
     <t>Aug 2023 -  Jul 2024 (22/23 learners) (26/03/26)</t>
   </si>
   <si>
@@ -156,6 +150,12 @@
   </si>
   <si>
     <t>April 2025 - Mar 2026 (TBC)</t>
+  </si>
+  <si>
+    <t>Apr 2026 (22/05/26)</t>
+  </si>
+  <si>
+    <t>May 2026 (June 2026)</t>
   </si>
 </sst>
 </file>
@@ -565,7 +565,7 @@
         <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="125" customHeight="1" x14ac:dyDescent="0.35">
@@ -579,7 +579,7 @@
         <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -593,7 +593,7 @@
         <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.35">
@@ -635,7 +635,7 @@
         <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -688,10 +688,10 @@
         <v>28</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -702,10 +702,10 @@
         <v>27</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="27" customHeight="1" x14ac:dyDescent="0.35">
@@ -716,10 +716,10 @@
         <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
UPdate to latest job ad data Delete unused files and folders
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7D70FA9-1DA0-472D-9218-E1429AD6A4EA}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D322B151-E5AF-44D5-BDD3-7EE764637753}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
@@ -152,10 +152,10 @@
     <t>April 2025 - Mar 2026 (TBC)</t>
   </si>
   <si>
-    <t>Apr 2026 (22/05/26)</t>
-  </si>
-  <si>
-    <t>May 2026 (June 2026)</t>
+    <t>May 2026 (26/06/26)</t>
+  </si>
+  <si>
+    <t>June 2026 (July 2026)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update to latest job advert data. Fix a few errors with the import sequencing. There is still an error in the job ads page - to be fixed.
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D322B151-E5AF-44D5-BDD3-7EE764637753}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{530D27F9-136A-455C-999C-FC6AECF97A39}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
@@ -152,10 +152,10 @@
     <t>April 2025 - Mar 2026 (TBC)</t>
   </si>
   <si>
-    <t>May 2026 (26/06/26)</t>
-  </si>
-  <si>
-    <t>June 2026 (July 2026)</t>
+    <t>Jun 2026 (24/07/26)</t>
+  </si>
+  <si>
+    <t>July 2026 (Aug 2026)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update to JUly 26 online job ads
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{530D27F9-136A-455C-999C-FC6AECF97A39}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DFE5B48-4D29-4031-B9C5-11DE375EC3CB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
@@ -152,10 +152,10 @@
     <t>April 2025 - Mar 2026 (TBC)</t>
   </si>
   <si>
-    <t>Jun 2026 (24/07/26)</t>
-  </si>
-  <si>
-    <t>July 2026 (Aug 2026)</t>
+    <t>Jul 2026 (21/08/26)</t>
+  </si>
+  <si>
+    <t>August 2026 (Sep 2026)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update to June 26 APS data
</commit_message>
<xml_diff>
--- a/Data/3-1_DataTable/DataTable.xlsx
+++ b/Data/3-1_DataTable/DataTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://educationgovuk-my.sharepoint.com/personal/paul_james_education_gov_uk/Documents/Documents/RProjects/lsip_dashboard/Data/3-1_DataTable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DFE5B48-4D29-4031-B9C5-11DE375EC3CB}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{BB966AC7-D478-46F4-96D8-4ADE6513DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DEE3EBA-6B8C-41C5-92E4-ED52225FAEF6}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
+    <workbookView xWindow="1820" yWindow="20" windowWidth="20660" windowHeight="14300" xr2:uid="{677CE7B9-0003-4845-87B7-4FABD7ACD82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
   <si>
     <t>Data​</t>
   </si>
@@ -156,6 +156,12 @@
   </si>
   <si>
     <t>August 2026 (Sep 2026)</t>
+  </si>
+  <si>
+    <t>April 2025 - Mar 2026 (Sep 26)</t>
+  </si>
+  <si>
+    <t>July 2025 - June 2026 (TBC)</t>
   </si>
 </sst>
 </file>
@@ -562,10 +568,10 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="125" customHeight="1" x14ac:dyDescent="0.35">
@@ -576,10 +582,10 @@
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -590,10 +596,10 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>